<commit_message>
adding new user is working properly
</commit_message>
<xml_diff>
--- a/backend/insertData/ActiveAttorneyRoster3.xlsx
+++ b/backend/insertData/ActiveAttorneyRoster3.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AC3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -534,6 +534,9 @@
       <c r="O2" t="str">
         <v>F</v>
       </c>
+      <c r="P2" t="str">
+        <v xml:space="preserve">No change </v>
+      </c>
       <c r="Q2" t="str">
         <v>narayangr@ewff.com</v>
       </c>
@@ -562,22 +565,102 @@
         <v>dkfbkjfbnugfbwnefhfnjnnen</v>
       </c>
       <c r="Z2" t="str">
-        <v>Yes</v>
+        <v>no</v>
       </c>
       <c r="AA2" t="str">
         <v>Yashaswini</v>
       </c>
       <c r="AB2" t="str">
-        <v>Tue Oct 22 2024 00:00:00 GMT+0530 (India Standard Time)</v>
+        <v>2024-10-21T18:30:00.000Z</v>
       </c>
       <c r="AC2" t="str">
+        <v>Yashaswini10003</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>4001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Darshan</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Mysore</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Mysore</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Mysore</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="H3" t="str">
+        <v>India</v>
+      </c>
+      <c r="I3" t="str">
+        <v>57-0989</v>
+      </c>
+      <c r="J3" t="str">
+        <v>6567890087</v>
+      </c>
+      <c r="K3" t="str">
+        <v>97656</v>
+      </c>
+      <c r="L3" t="str">
+        <v>uhjgjvb</v>
+      </c>
+      <c r="M3" t="str">
+        <v>gh87</v>
+      </c>
+      <c r="N3" t="str">
+        <v>7h</v>
+      </c>
+      <c r="O3" t="str">
+        <v>yvhb nm</v>
+      </c>
+      <c r="P3" t="str">
+        <v>uigbij</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>kv .nm</v>
+      </c>
+      <c r="R3" t="str">
+        <v xml:space="preserve">bhm </v>
+      </c>
+      <c r="S3" t="str">
+        <v>l/bxm</v>
+      </c>
+      <c r="T3" t="str">
+        <v>bnn</v>
+      </c>
+      <c r="U3" t="str">
+        <v>n</v>
+      </c>
+      <c r="W3" t="str">
+        <v>n</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>n</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>n</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Yashaswini</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>2025-01-01T00:00:00.000Z</v>
+      </c>
+      <c r="AC3" t="str">
         <v>Yashaswini10003</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>